<commit_message>
feat(ventas): columna "No. Factura" (referencia) en plantilla de ventas
Agrega columna informativa de número(s) de factura a la plantilla
"Ventas por Vendedor". Es solo referencia para conciliación: el parser
la ignora (mapea por nombre de columna) y el sistema no la guarda.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/plantilla_ventas.xlsx
+++ b/public/templates/plantilla_ventas.xlsx
@@ -398,15 +398,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:H3"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
     <col min="3" max="3" width="32.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
     <col min="5" max="5" width="14.83203125" customWidth="1"/>
     <col min="6" max="6" width="14.83203125" customWidth="1"/>
     <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -420,15 +421,18 @@
         <v>Nombre Comercial</v>
       </c>
       <c r="D1" t="str">
+        <v>No. Factura</v>
+      </c>
+      <c r="E1" t="str">
         <v>Venta Bruta</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Neto</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Descuento</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Neto-Desc</v>
       </c>
     </row>
@@ -442,16 +446,19 @@
       <c r="C2" t="str">
         <v>HOTEL EJEMPLO SA DE CV</v>
       </c>
-      <c r="D2">
-        <v>12500</v>
+      <c r="D2" t="str">
+        <v>A1234, A1290</v>
       </c>
       <c r="E2">
         <v>12500</v>
       </c>
       <c r="F2">
+        <v>12500</v>
+      </c>
+      <c r="G2">
         <v>0</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>12500</v>
       </c>
     </row>
@@ -465,29 +472,32 @@
       <c r="C3" t="str">
         <v>RESTAURANTE DEMO</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="str">
+        <v>A1305</v>
+      </c>
+      <c r="E3">
         <v>8400.5</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>9744.58</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>1344.08</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>8400.5</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A22"/>
   <cols>
     <col min="1" max="1" width="115.83203125" customWidth="1"/>
   </cols>
@@ -549,57 +559,62 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Venta Bruta       Monto de venta bruta del mes. Alimenta el total de ventas y el ranking.</v>
+        <v>No. Factura       Opcional, SOLO REFERENCIA. Anota aquí la(s) factura(s) del mes (sepáralas con comas). El sistema NO la guarda; sirve para tu control y conciliación.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Neto              Opcional. Importe neto antes de descuento.</v>
+        <v>Venta Bruta       Monto de venta bruta del mes. Alimenta el total de ventas y el ranking.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Descuento         Opcional. Descuento aplicado.</v>
+        <v>Neto              Opcional. Importe neto antes de descuento.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Neto-Desc         Opcional. Neto después de descuento.</v>
+        <v>Descuento         Opcional. Descuento aplicado.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v/>
+        <v>Neto-Desc         Opcional. Neto después de descuento.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Emparejamiento: # Cliente CONTPAQi → cuenta del CRM → vendedor asignado.</v>
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Si una cuenta no existe en el CRM o no tiene vendedor asignado, esa fila se reporta como error y no se importa.</v>
+        <v>Emparejamiento: # Cliente CONTPAQi → cuenta del CRM → vendedor asignado.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Re-importar el mismo mes ACTUALIZA los datos de ese cliente (upsert por cuenta + periodo).</v>
+        <v>Si una cuenta no existe en el CRM o no tiene vendedor asignado, esa fila se reporta como error y no se importa.</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v/>
+        <v>Re-importar el mismo mes ACTUALIZA los datos de ese cliente (upsert por cuenta + periodo).</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
         <v>¿Tienes el reporte crudo de CONTPAQ con detalle por producto? Súbelo tal cual — es el formato recomendado y NO necesita esta plantilla.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A22"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(ventas): columna "No. Factura" (referencia) en plantilla de ventas (#90)
Agrega columna informativa de número(s) de factura a la plantilla
"Ventas por Vendedor". Es solo referencia para conciliación: el parser
la ignora (mapea por nombre de columna) y el sistema no la guarda.

Co-authored-by: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/plantilla_ventas.xlsx
+++ b/public/templates/plantilla_ventas.xlsx
@@ -398,15 +398,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:H3"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
     <col min="3" max="3" width="32.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
     <col min="5" max="5" width="14.83203125" customWidth="1"/>
     <col min="6" max="6" width="14.83203125" customWidth="1"/>
     <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -420,15 +421,18 @@
         <v>Nombre Comercial</v>
       </c>
       <c r="D1" t="str">
+        <v>No. Factura</v>
+      </c>
+      <c r="E1" t="str">
         <v>Venta Bruta</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Neto</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Descuento</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Neto-Desc</v>
       </c>
     </row>
@@ -442,16 +446,19 @@
       <c r="C2" t="str">
         <v>HOTEL EJEMPLO SA DE CV</v>
       </c>
-      <c r="D2">
-        <v>12500</v>
+      <c r="D2" t="str">
+        <v>A1234, A1290</v>
       </c>
       <c r="E2">
         <v>12500</v>
       </c>
       <c r="F2">
+        <v>12500</v>
+      </c>
+      <c r="G2">
         <v>0</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>12500</v>
       </c>
     </row>
@@ -465,29 +472,32 @@
       <c r="C3" t="str">
         <v>RESTAURANTE DEMO</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="str">
+        <v>A1305</v>
+      </c>
+      <c r="E3">
         <v>8400.5</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>9744.58</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>1344.08</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>8400.5</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A22"/>
   <cols>
     <col min="1" max="1" width="115.83203125" customWidth="1"/>
   </cols>
@@ -549,57 +559,62 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Venta Bruta       Monto de venta bruta del mes. Alimenta el total de ventas y el ranking.</v>
+        <v>No. Factura       Opcional, SOLO REFERENCIA. Anota aquí la(s) factura(s) del mes (sepáralas con comas). El sistema NO la guarda; sirve para tu control y conciliación.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Neto              Opcional. Importe neto antes de descuento.</v>
+        <v>Venta Bruta       Monto de venta bruta del mes. Alimenta el total de ventas y el ranking.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Descuento         Opcional. Descuento aplicado.</v>
+        <v>Neto              Opcional. Importe neto antes de descuento.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Neto-Desc         Opcional. Neto después de descuento.</v>
+        <v>Descuento         Opcional. Descuento aplicado.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v/>
+        <v>Neto-Desc         Opcional. Neto después de descuento.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Emparejamiento: # Cliente CONTPAQi → cuenta del CRM → vendedor asignado.</v>
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Si una cuenta no existe en el CRM o no tiene vendedor asignado, esa fila se reporta como error y no se importa.</v>
+        <v>Emparejamiento: # Cliente CONTPAQi → cuenta del CRM → vendedor asignado.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Re-importar el mismo mes ACTUALIZA los datos de ese cliente (upsert por cuenta + periodo).</v>
+        <v>Si una cuenta no existe en el CRM o no tiene vendedor asignado, esa fila se reporta como error y no se importa.</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v/>
+        <v>Re-importar el mismo mes ACTUALIZA los datos de ese cliente (upsert por cuenta + periodo).</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
         <v>¿Tienes el reporte crudo de CONTPAQ con detalle por producto? Súbelo tal cual — es el formato recomendado y NO necesita esta plantilla.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A22"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>